<commit_message>
Feat: Employee Payroll, Payslip History & Mandant Config (v3.1)
</commit_message>
<xml_diff>
--- a/backend/Mandanten/Elektroniker_Testbetrieb/Einnahmen/einnahmen.xlsx
+++ b/backend/Mandanten/Elektroniker_Testbetrieb/Einnahmen/einnahmen.xlsx
@@ -445,13 +445,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="15" customWidth="1" min="6" max="6"/>
     <col width="10" customWidth="1" min="7" max="7"/>
@@ -568,6 +568,43 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>2026-001</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>02.01.2026</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Oma_Erna</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>1.0 Stk x NYM-J Kabel 3x1,5 (EP: 1.50€), 1.0 Std x Meisterstunde (EP: 75.00€), 1.0 Stk x Anfahrt pauschal (EP: 35.00€)</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>111.50</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>132.69</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Offen</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>